<commit_message>
update and removed a test case
</commit_message>
<xml_diff>
--- a/data-files/users.xlsx
+++ b/data-files/users.xlsx
@@ -19,22 +19,22 @@
     <t>password</t>
   </si>
   <si>
-    <t>u1_1775633644001_32971</t>
-  </si>
-  <si>
-    <t>Pass@1775633644001_32971</t>
-  </si>
-  <si>
-    <t>u2_1775633644001_99301</t>
-  </si>
-  <si>
-    <t>Pass@1775633644001_99301</t>
-  </si>
-  <si>
-    <t>u3_1775633644001_76910</t>
-  </si>
-  <si>
-    <t>Pass@1775633644001_76910</t>
+    <t>u1_1775644757664_24461</t>
+  </si>
+  <si>
+    <t>Pass@1775644757664_24461</t>
+  </si>
+  <si>
+    <t>u2_1775644757664_7727</t>
+  </si>
+  <si>
+    <t>Pass@1775644757664_7727</t>
+  </si>
+  <si>
+    <t>u3_1775644757664_93374</t>
+  </si>
+  <si>
+    <t>Pass@1775644757664_93374</t>
   </si>
 </sst>
 </file>

</xml_diff>